<commit_message>
Show the input workbooks and how the settings describe them
plot_sheet draws a worksheet as it looks in Excel (column letters, row numbers,
fill colours including theme tints, values, merged cells, rotated text), from the
file itself. The two examples now follow the steps of a real project: look at the
input workbook, describe it in the settings, run. README: the settings describe
how each workbook is organised; per example, pictures of the input sheets, a table
pairing workbook features with settings, and the first rows of the output tables.
Ratings columns that hold only whole numbers stay whole (69, not 69.0).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_2_one_sheet_per_trial.xlsx
+++ b/examples/data/example_2_one_sheet_per_trial.xlsx
@@ -1120,6 +1120,10 @@
   </sheetPr>
   <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1522,6 +1526,10 @@
   </sheetPr>
   <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1860,6 +1868,10 @@
   </sheetPr>
   <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2582,6 +2594,10 @@
   </sheetPr>
   <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Read notes written outside the tables (sheet_values)
Single values typed next to a label on a sheet - on a field map (site, cultivar,
planting date) or above a ratings table (growth stage, application date) - become
columns: of the design table for layouts, of the ratings for rating sources (read
on every assessment sheet; an assessment can add or replace fields). A field is
found by its label (value in the first filled cell to the right, or below) or by
its cell address. Example 2 shows both. README: which columns of a ratings sheet
are kept and which are left out, and the new setting.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_2_one_sheet_per_trial.xlsx
+++ b/examples/data/example_2_one_sheet_per_trial.xlsx
@@ -463,6 +463,28 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Site:</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Example farm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Cultivar:</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Cultivar X</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="B3" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
sheet_values left/above; matching figure sizes; readable distribution charts
- sheet_values: a value can also be left of or above its label.
- plot_distribution: font_size setting (bands grow with the text); the legend band
  follows the number of legend rows.
- Examples: input pictures of the same height side by side; Example 2 with narrow
  columns and tall plot rows, its figures the same size as Example 1's; smaller
  distribution charts with larger text, left-aligned in the README.
- README: picture of the notes read by sheet_values and the columns they become.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_2_one_sheet_per_trial.xlsx
+++ b/examples/data/example_2_one_sheet_per_trial.xlsx
@@ -455,6 +455,34 @@
   </sheetPr>
   <dimension ref="B1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="18" max="18"/>
+    <col width="5" customWidth="1" min="19" max="19"/>
+    <col width="5" customWidth="1" min="20" max="20"/>
+    <col width="5" customWidth="1" min="21" max="21"/>
+    <col width="5" customWidth="1" min="22" max="22"/>
+    <col width="5" customWidth="1" min="23" max="23"/>
+    <col width="5" customWidth="1" min="24" max="24"/>
+    <col width="5" customWidth="1" min="25" max="25"/>
+    <col width="5" customWidth="1" min="26" max="26"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
@@ -507,7 +535,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="39.375" customHeight="1">
       <c r="B4" s="2" t="n">
         <v>40</v>
       </c>
@@ -584,7 +612,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="39.375" customHeight="1">
       <c r="B5" s="2" t="n">
         <v>31</v>
       </c>
@@ -661,7 +689,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="39.375" customHeight="1">
       <c r="B6" s="2" t="n">
         <v>30</v>
       </c>
@@ -738,7 +766,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="39.375" customHeight="1">
       <c r="B7" s="2" t="n">
         <v>21</v>
       </c>
@@ -815,7 +843,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="39.375" customHeight="1">
       <c r="B8" s="2" t="n">
         <v>20</v>
       </c>
@@ -892,7 +920,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="39.375" customHeight="1">
       <c r="B9" s="2" t="n">
         <v>11</v>
       </c>
@@ -969,7 +997,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="39.375" customHeight="1">
       <c r="B10" s="2" t="n">
         <v>10</v>
       </c>
@@ -1046,7 +1074,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="39.375" customHeight="1">
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Tighter distribution charts; example 2 map shows where the field ends
- plot_distribution measures the date labels and the legend after drawing
  and sizes the left and bottom space to fit them (a legend_height that is
  set explicitly is still used as given)
- example distribution charts 8.5 in wide; README shows them at 62%
- example 2: the field_map picture includes the empty row 12 below the
  plots; plot rows are 37.5 pt so the picture keeps its height

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/data/example_2_one_sheet_per_trial.xlsx
+++ b/examples/data/example_2_one_sheet_per_trial.xlsx
@@ -535,7 +535,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="39.375" customHeight="1">
+    <row r="4" ht="37.5" customHeight="1">
       <c r="B4" s="2" t="n">
         <v>40</v>
       </c>
@@ -612,7 +612,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" ht="39.375" customHeight="1">
+    <row r="5" ht="37.5" customHeight="1">
       <c r="B5" s="2" t="n">
         <v>31</v>
       </c>
@@ -689,7 +689,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" ht="39.375" customHeight="1">
+    <row r="6" ht="37.5" customHeight="1">
       <c r="B6" s="2" t="n">
         <v>30</v>
       </c>
@@ -766,7 +766,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" ht="39.375" customHeight="1">
+    <row r="7" ht="37.5" customHeight="1">
       <c r="B7" s="2" t="n">
         <v>21</v>
       </c>
@@ -843,7 +843,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" ht="39.375" customHeight="1">
+    <row r="8" ht="37.5" customHeight="1">
       <c r="B8" s="2" t="n">
         <v>20</v>
       </c>
@@ -920,7 +920,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" ht="39.375" customHeight="1">
+    <row r="9" ht="37.5" customHeight="1">
       <c r="B9" s="2" t="n">
         <v>11</v>
       </c>
@@ -997,7 +997,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" ht="39.375" customHeight="1">
+    <row r="10" ht="37.5" customHeight="1">
       <c r="B10" s="2" t="n">
         <v>10</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" ht="39.375" customHeight="1">
+    <row r="11" ht="37.5" customHeight="1">
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>

</xml_diff>